<commit_message>
BRO object SAD added, others updated
Added format for BRO object Site Assessment Data (SAD), updated others
</commit_message>
<xml_diff>
--- a/Booronderzoek (BHR)/BROObject - BHRGT description datafile NL (v0.8).xlsx
+++ b/Booronderzoek (BHR)/BROObject - BHRGT description datafile NL (v0.8).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://3hydro-my.sharepoint.com/personal/jos_von_asmuth_3hydro_nl/Documents/MATLAB/Menyanthes/DocumentenSVN/Bron- en BRO-data/BRO-Spreadsheet-en-tabelformat/Booronderzoek (BHR)/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://3hydro-my.sharepoint.com/personal/jos_von_asmuth_3hydro_nl/Documents/GitHub/QC-Protocol/BRO-Spreadsheet-en-tabelformat/Booronderzoek (BHR)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="188" documentId="8_{9D121EB8-C1B7-4D82-96BC-5623D013166D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C9F5918-3A6A-4942-ADF5-5B5504E30DB8}"/>
+  <xr:revisionPtr revIDLastSave="191" documentId="8_{9D121EB8-C1B7-4D82-96BC-5623D013166D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{620DCC2C-1F2C-4376-9122-AB9E305908FF}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{26814B37-6F38-4D5A-99CF-A0A5CD7480CB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{26814B37-6F38-4D5A-99CF-A0A5CD7480CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Toelichting" sheetId="8" r:id="rId1"/>
@@ -1659,7 +1659,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1782,7 +1782,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="17" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2455,13 +2454,13 @@
   <sheetFormatPr defaultColWidth="16.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="20" bestFit="1" customWidth="1"/>
@@ -2472,12 +2471,12 @@
     <col min="17" max="17" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="27" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="24" bestFit="1" customWidth="1"/>
+    <col min="25" max="27" width="24.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
@@ -3292,62 +3291,62 @@
     <col min="20" max="16384" width="9.140625" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="46" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="47" t="s">
+    <row r="1" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="47" t="s">
         <v>102</v>
       </c>
-      <c r="C1" s="48" t="s">
+      <c r="C1" s="47" t="s">
         <v>99</v>
       </c>
-      <c r="D1" s="48" t="s">
+      <c r="D1" s="47" t="s">
         <v>86</v>
       </c>
-      <c r="E1" s="48" t="s">
+      <c r="E1" s="47" t="s">
         <v>83</v>
       </c>
-      <c r="F1" s="48" t="s">
+      <c r="F1" s="47" t="s">
         <v>100</v>
       </c>
-      <c r="G1" s="48" t="s">
+      <c r="G1" s="47" t="s">
         <v>82</v>
       </c>
-      <c r="H1" s="48" t="s">
+      <c r="H1" s="47" t="s">
         <v>250</v>
       </c>
-      <c r="I1" s="48" t="s">
+      <c r="I1" s="47" t="s">
         <v>74</v>
       </c>
-      <c r="J1" s="48" t="s">
+      <c r="J1" s="47" t="s">
         <v>101</v>
       </c>
-      <c r="K1" s="48" t="s">
+      <c r="K1" s="47" t="s">
         <v>75</v>
       </c>
-      <c r="L1" s="48" t="s">
+      <c r="L1" s="47" t="s">
         <v>86</v>
       </c>
-      <c r="M1" s="48" t="s">
+      <c r="M1" s="47" t="s">
         <v>69</v>
       </c>
-      <c r="N1" s="48" t="s">
+      <c r="N1" s="47" t="s">
         <v>71</v>
       </c>
-      <c r="O1" s="48" t="s">
+      <c r="O1" s="47" t="s">
         <v>85</v>
       </c>
-      <c r="P1" s="48" t="s">
+      <c r="P1" s="47" t="s">
         <v>81</v>
       </c>
-      <c r="Q1" s="48" t="s">
+      <c r="Q1" s="47" t="s">
         <v>88</v>
       </c>
-      <c r="R1" s="48" t="s">
+      <c r="R1" s="47" t="s">
         <v>90</v>
       </c>
-      <c r="S1" s="49" t="s">
+      <c r="S1" s="48" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>